<commit_message>
Add three Telegram emoji: link, GitHub, info; update navigation and catalog
</commit_message>
<xml_diff>
--- a/MOKO/00_Каталог_файлов.xlsx
+++ b/MOKO/00_Каталог_файлов.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -716,6 +716,23 @@
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Ссылки на файлы работают при скачивании папки MOKO с сохранением структуры.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Telegram — 3 новых эмодзи: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/MOKO_3_эмодзи_Просмотр.html</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Вместе с прежними 24 теперь 27. Исходный комплект 24 не изменён.</t>
         </is>
       </c>
     </row>
@@ -746,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K741"/>
+  <dimension ref="A1:K755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -36894,6 +36911,611 @@
       </c>
       <c r="J741" s="5" t="inlineStr"/>
       <c r="K741" s="5" t="inlineStr"/>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>25_link</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/png_100/25_link.png</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I742" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>26_github</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/png_100/26_github.png</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I743" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>27_info</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/png_100/27_info.png</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I744" t="n">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>25_link</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/webp_100/25_link.webp</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I745" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>26_github</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/webp_100/26_github.webp</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I746" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>27_info</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/webp_100/27_info.webp</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I747" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>25_link</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/svg/25_link.svg</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I748" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>26_github</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/svg/26_github.svg</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I749" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>27_info</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/svg/27_info.svg</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I750" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>MOKO_3_эмодзи_Просмотр</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/MOKO_3_эмодзи_Просмотр.html</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I751" t="n">
+        <v>162.5</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>MOKO_3_эмодзи_Превью</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>JPG</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/MOKO_3_эмодзи_Превью.jpg</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I752" t="n">
+        <v>94.09999999999999</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>Привязка_эмодзи</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/Привязка_эмодзи.csv</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I753" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>README</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>TXT</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/README.md</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I754" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Эмодзи — дополнение: Ссылка, GitHub, Информация</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Дополнение на согласование</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>MOKO_3_эмодзи_дополнение_v02</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Дополнение_3/MOKO_3_эмодзи_дополнение_v02.zip</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I755" t="n">
+        <v>247.1</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K741"/>
@@ -37638,6 +38260,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H739" r:id="rId738"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H740" r:id="rId739"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H741" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H742" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H743" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H744" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H745" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H746" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H747" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H748" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H749" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H750" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H751" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H752" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H753" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H754" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H755" r:id="rId754"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 18-emoji set for the main Telegram group; refresh navigation and catalog
</commit_message>
<xml_diff>
--- a/MOKO/00_Каталог_файлов.xlsx
+++ b/MOKO/00_Каталог_файлов.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Файлы" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Файлы'!$A$1:$K$670</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Файлы'!$A$1:$K$729</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -718,8 +718,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K670"/>
+  <dimension ref="A1:K729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -32538,8 +32551,2638 @@
         <v>1.1</v>
       </c>
     </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>01_about</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/01_about.png</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I671" t="n">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>01_about</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/01_about.webp</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I672" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>01_about</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/01_about.svg</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I673" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>02_news</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/02_news.png</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I674" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>02_news</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/02_news.webp</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I675" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>02_news</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/02_news.svg</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I676" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>03_forum</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/03_forum.png</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I677" t="n">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>03_forum</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/03_forum.webp</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I678" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>03_forum</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/03_forum.svg</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I679" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>04_soft</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/04_soft.png</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I680" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>04_soft</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/04_soft.webp</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I681" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>04_soft</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/04_soft.svg</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I682" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>05_docs</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/05_docs.png</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I683" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>05_docs</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/05_docs.webp</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I684" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>05_docs</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/05_docs.svg</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I685" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>06_lifehack</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/06_lifehack.png</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I686" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>06_lifehack</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/06_lifehack.webp</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I687" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>06_lifehack</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/06_lifehack.svg</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I688" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>07_projects</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/07_projects.png</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I689" t="n">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>07_projects</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/07_projects.webp</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I690" t="n">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>07_projects</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/07_projects.svg</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I691" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>08_books</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/08_books.png</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I692" t="n">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>08_books</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/08_books.webp</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I693" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>08_books</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/08_books.svg</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I694" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>09_gallery</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/09_gallery.png</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I695" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>09_gallery</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/09_gallery.webp</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I696" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>09_gallery</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/09_gallery.svg</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I697" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>10_drivers</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/10_drivers.png</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I698" t="n">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>10_drivers</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/10_drivers.webp</t>
+        </is>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I699" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>10_drivers</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/10_drivers.svg</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I700" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>11_suggest</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/11_suggest.png</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I701" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>11_suggest</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/11_suggest.webp</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I702" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>11_suggest</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/11_suggest.svg</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I703" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>12_code</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/12_code.png</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I704" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>12_code</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/12_code.webp</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I705" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>12_code</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/12_code.svg</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I706" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>13_video</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/13_video.png</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I707" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>13_video</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/13_video.webp</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I708" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>13_video</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/13_video.svg</t>
+        </is>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I709" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>14_archive</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/14_archive.png</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I710" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>14_archive</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/14_archive.webp</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I711" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>14_archive</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/14_archive.svg</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I712" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>15_live</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/15_live.png</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I713" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>15_live</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/15_live.webp</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I714" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>15_live</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/15_live.svg</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I715" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>16_question</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/16_question.png</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I716" t="n">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>16_question</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/16_question.webp</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I717" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>16_question</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/16_question.svg</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I718" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>17_tests</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/17_tests.png</t>
+        </is>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I719" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>17_tests</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/17_tests.webp</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I720" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>17_tests</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/17_tests.svg</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I721" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>18_moko_se</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/png_100/18_moko_se.png</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I722" t="n">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>18_moko_se</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>WEBP</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>100 × 100</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/webp_100/18_moko_se.webp</t>
+        </is>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I723" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>18_moko_se</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>вектор</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/svg/18_moko_se.svg</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I724" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>набор 18 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>MOKO_18_эмодзи_группа_v01</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/MOKO_18_эмодзи_группа_v01.zip</t>
+        </is>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I725" t="n">
+        <v>573.5</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>MOKO_Группа_Просмотр</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/MOKO_Группа_Просмотр.html</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I726" t="n">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>MOKO_Группа_Превью</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>JPG</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/MOKO_Группа_Превью.jpg</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I727" t="n">
+        <v>182.1</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>Привязка_эмодзи_группы</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/Привязка_эмодзи_группы.csv</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I728" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Эмодзи главной группы</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>добавлено 18.09.2026 · не опубликовано</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>README</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>TXT</t>
+        </is>
+      </c>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/README.md</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>Открыть</t>
+        </is>
+      </c>
+      <c r="I729" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K670"/>
+  <autoFilter ref="A1:K729"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
@@ -33210,6 +35853,65 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H668" r:id="rId667"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H669" r:id="rId668"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H670" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H671" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H672" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H673" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H674" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H675" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H676" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H677" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H678" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H679" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H680" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H681" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H682" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H683" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H684" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H685" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H686" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H687" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H688" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H689" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H690" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H691" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H692" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H693" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H694" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H695" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H696" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H697" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H698" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H699" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H700" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H701" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H702" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H703" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H704" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H705" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H706" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H707" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H708" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H709" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H710" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H711" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H712" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H713" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H714" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H715" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H716" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H717" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H718" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H719" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H720" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H721" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H722" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H723" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H724" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H725" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H726" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H727" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H728" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H729" r:id="rId728"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Group emoji v02: bigger filled recognizable glyphs
</commit_message>
<xml_diff>
--- a/MOKO/00_Каталог_файлов.xlsx
+++ b/MOKO/00_Каталог_файлов.xlsx
@@ -32564,7 +32564,7 @@
       </c>
       <c r="C671" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D671" t="inlineStr">
@@ -32593,7 +32593,7 @@
         </is>
       </c>
       <c r="I671" t="n">
-        <v>8.300000000000001</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="672">
@@ -32609,7 +32609,7 @@
       </c>
       <c r="C672" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D672" t="inlineStr">
@@ -32638,7 +32638,7 @@
         </is>
       </c>
       <c r="I672" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="673">
@@ -32654,7 +32654,7 @@
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
@@ -32683,7 +32683,7 @@
         </is>
       </c>
       <c r="I673" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="674">
@@ -32699,7 +32699,7 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D674" t="inlineStr">
@@ -32728,7 +32728,7 @@
         </is>
       </c>
       <c r="I674" t="n">
-        <v>7.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="675">
@@ -32744,7 +32744,7 @@
       </c>
       <c r="C675" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D675" t="inlineStr">
@@ -32773,7 +32773,7 @@
         </is>
       </c>
       <c r="I675" t="n">
-        <v>4.2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="676">
@@ -32789,7 +32789,7 @@
       </c>
       <c r="C676" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D676" t="inlineStr">
@@ -32818,7 +32818,7 @@
         </is>
       </c>
       <c r="I676" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="677">
@@ -32834,7 +32834,7 @@
       </c>
       <c r="C677" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D677" t="inlineStr">
@@ -32863,7 +32863,7 @@
         </is>
       </c>
       <c r="I677" t="n">
-        <v>8.699999999999999</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="678">
@@ -32879,7 +32879,7 @@
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D678" t="inlineStr">
@@ -32908,7 +32908,7 @@
         </is>
       </c>
       <c r="I678" t="n">
-        <v>4.7</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="679">
@@ -32924,7 +32924,7 @@
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D679" t="inlineStr">
@@ -32953,7 +32953,7 @@
         </is>
       </c>
       <c r="I679" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="680">
@@ -32969,7 +32969,7 @@
       </c>
       <c r="C680" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D680" t="inlineStr">
@@ -32998,7 +32998,7 @@
         </is>
       </c>
       <c r="I680" t="n">
-        <v>9</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="681">
@@ -33014,7 +33014,7 @@
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D681" t="inlineStr">
@@ -33043,7 +33043,7 @@
         </is>
       </c>
       <c r="I681" t="n">
-        <v>5.1</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="682">
@@ -33059,7 +33059,7 @@
       </c>
       <c r="C682" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D682" t="inlineStr">
@@ -33088,7 +33088,7 @@
         </is>
       </c>
       <c r="I682" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="683">
@@ -33104,7 +33104,7 @@
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D683" t="inlineStr">
@@ -33133,7 +33133,7 @@
         </is>
       </c>
       <c r="I683" t="n">
-        <v>7.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="684">
@@ -33149,7 +33149,7 @@
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D684" t="inlineStr">
@@ -33178,7 +33178,7 @@
         </is>
       </c>
       <c r="I684" t="n">
-        <v>4.3</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="685">
@@ -33194,7 +33194,7 @@
       </c>
       <c r="C685" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D685" t="inlineStr">
@@ -33223,7 +33223,7 @@
         </is>
       </c>
       <c r="I685" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="686">
@@ -33239,7 +33239,7 @@
       </c>
       <c r="C686" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D686" t="inlineStr">
@@ -33268,7 +33268,7 @@
         </is>
       </c>
       <c r="I686" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="687">
@@ -33284,7 +33284,7 @@
       </c>
       <c r="C687" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D687" t="inlineStr">
@@ -33313,7 +33313,7 @@
         </is>
       </c>
       <c r="I687" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="688">
@@ -33329,7 +33329,7 @@
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D688" t="inlineStr">
@@ -33358,7 +33358,7 @@
         </is>
       </c>
       <c r="I688" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="689">
@@ -33374,7 +33374,7 @@
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
@@ -33403,7 +33403,7 @@
         </is>
       </c>
       <c r="I689" t="n">
-        <v>10.6</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="690">
@@ -33419,7 +33419,7 @@
       </c>
       <c r="C690" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D690" t="inlineStr">
@@ -33448,7 +33448,7 @@
         </is>
       </c>
       <c r="I690" t="n">
-        <v>5.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="691">
@@ -33464,7 +33464,7 @@
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
@@ -33493,7 +33493,7 @@
         </is>
       </c>
       <c r="I691" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="692">
@@ -33509,7 +33509,7 @@
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D692" t="inlineStr">
@@ -33538,7 +33538,7 @@
         </is>
       </c>
       <c r="I692" t="n">
-        <v>9.1</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="693">
@@ -33554,7 +33554,7 @@
       </c>
       <c r="C693" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D693" t="inlineStr">
@@ -33583,7 +33583,7 @@
         </is>
       </c>
       <c r="I693" t="n">
-        <v>5.1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="694">
@@ -33599,7 +33599,7 @@
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D694" t="inlineStr">
@@ -33628,7 +33628,7 @@
         </is>
       </c>
       <c r="I694" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="695">
@@ -33644,7 +33644,7 @@
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D695" t="inlineStr">
@@ -33673,7 +33673,7 @@
         </is>
       </c>
       <c r="I695" t="n">
-        <v>8</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="696">
@@ -33689,7 +33689,7 @@
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
@@ -33718,7 +33718,7 @@
         </is>
       </c>
       <c r="I696" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="697">
@@ -33734,7 +33734,7 @@
       </c>
       <c r="C697" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D697" t="inlineStr">
@@ -33763,7 +33763,7 @@
         </is>
       </c>
       <c r="I697" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="698">
@@ -33779,7 +33779,7 @@
       </c>
       <c r="C698" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D698" t="inlineStr">
@@ -33808,7 +33808,7 @@
         </is>
       </c>
       <c r="I698" t="n">
-        <v>8.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="699">
@@ -33824,7 +33824,7 @@
       </c>
       <c r="C699" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D699" t="inlineStr">
@@ -33853,7 +33853,7 @@
         </is>
       </c>
       <c r="I699" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="700">
@@ -33869,7 +33869,7 @@
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D700" t="inlineStr">
@@ -33898,7 +33898,7 @@
         </is>
       </c>
       <c r="I700" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="701">
@@ -33914,7 +33914,7 @@
       </c>
       <c r="C701" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D701" t="inlineStr">
@@ -33943,7 +33943,7 @@
         </is>
       </c>
       <c r="I701" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="702">
@@ -33959,7 +33959,7 @@
       </c>
       <c r="C702" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D702" t="inlineStr">
@@ -33988,7 +33988,7 @@
         </is>
       </c>
       <c r="I702" t="n">
-        <v>4.6</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="703">
@@ -34004,7 +34004,7 @@
       </c>
       <c r="C703" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D703" t="inlineStr">
@@ -34033,7 +34033,7 @@
         </is>
       </c>
       <c r="I703" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="704">
@@ -34049,7 +34049,7 @@
       </c>
       <c r="C704" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D704" t="inlineStr">
@@ -34078,7 +34078,7 @@
         </is>
       </c>
       <c r="I704" t="n">
-        <v>7.6</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="705">
@@ -34094,7 +34094,7 @@
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D705" t="inlineStr">
@@ -34123,7 +34123,7 @@
         </is>
       </c>
       <c r="I705" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="706">
@@ -34139,7 +34139,7 @@
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D706" t="inlineStr">
@@ -34168,7 +34168,7 @@
         </is>
       </c>
       <c r="I706" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="707">
@@ -34184,7 +34184,7 @@
       </c>
       <c r="C707" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D707" t="inlineStr">
@@ -34213,7 +34213,7 @@
         </is>
       </c>
       <c r="I707" t="n">
-        <v>8</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="708">
@@ -34229,7 +34229,7 @@
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D708" t="inlineStr">
@@ -34258,7 +34258,7 @@
         </is>
       </c>
       <c r="I708" t="n">
-        <v>4.7</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="709">
@@ -34274,7 +34274,7 @@
       </c>
       <c r="C709" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D709" t="inlineStr">
@@ -34303,7 +34303,7 @@
         </is>
       </c>
       <c r="I709" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="710">
@@ -34319,7 +34319,7 @@
       </c>
       <c r="C710" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D710" t="inlineStr">
@@ -34348,7 +34348,7 @@
         </is>
       </c>
       <c r="I710" t="n">
-        <v>7.6</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="711">
@@ -34364,7 +34364,7 @@
       </c>
       <c r="C711" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D711" t="inlineStr">
@@ -34393,7 +34393,7 @@
         </is>
       </c>
       <c r="I711" t="n">
-        <v>4.2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="712">
@@ -34409,7 +34409,7 @@
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D712" t="inlineStr">
@@ -34438,7 +34438,7 @@
         </is>
       </c>
       <c r="I712" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="713">
@@ -34454,7 +34454,7 @@
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
@@ -34483,7 +34483,7 @@
         </is>
       </c>
       <c r="I713" t="n">
-        <v>9.300000000000001</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="714">
@@ -34499,7 +34499,7 @@
       </c>
       <c r="C714" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D714" t="inlineStr">
@@ -34528,7 +34528,7 @@
         </is>
       </c>
       <c r="I714" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="715">
@@ -34544,7 +34544,7 @@
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
@@ -34573,7 +34573,7 @@
         </is>
       </c>
       <c r="I715" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="716">
@@ -34589,7 +34589,7 @@
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
@@ -34618,7 +34618,7 @@
         </is>
       </c>
       <c r="I716" t="n">
-        <v>8.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="717">
@@ -34634,7 +34634,7 @@
       </c>
       <c r="C717" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D717" t="inlineStr">
@@ -34663,7 +34663,7 @@
         </is>
       </c>
       <c r="I717" t="n">
-        <v>4.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="718">
@@ -34679,7 +34679,7 @@
       </c>
       <c r="C718" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D718" t="inlineStr">
@@ -34708,7 +34708,7 @@
         </is>
       </c>
       <c r="I718" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="719">
@@ -34724,7 +34724,7 @@
       </c>
       <c r="C719" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D719" t="inlineStr">
@@ -34753,7 +34753,7 @@
         </is>
       </c>
       <c r="I719" t="n">
-        <v>9.199999999999999</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="720">
@@ -34769,7 +34769,7 @@
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
@@ -34798,7 +34798,7 @@
         </is>
       </c>
       <c r="I720" t="n">
-        <v>5.4</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="721">
@@ -34814,7 +34814,7 @@
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D721" t="inlineStr">
@@ -34843,7 +34843,7 @@
         </is>
       </c>
       <c r="I721" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="722">
@@ -34859,7 +34859,7 @@
       </c>
       <c r="C722" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D722" t="inlineStr">
@@ -34888,7 +34888,7 @@
         </is>
       </c>
       <c r="I722" t="n">
-        <v>7.8</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="723">
@@ -34904,7 +34904,7 @@
       </c>
       <c r="C723" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D723" t="inlineStr">
@@ -34933,7 +34933,7 @@
         </is>
       </c>
       <c r="I723" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="724">
@@ -34949,7 +34949,7 @@
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
@@ -34978,7 +34978,7 @@
         </is>
       </c>
       <c r="I724" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="725">
@@ -34994,12 +34994,12 @@
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>набор 18 · не опубликовано</t>
+          <t>набор 18 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>MOKO_18_эмодзи_группа_v01</t>
+          <t>MOKO_18_эмодзи_группа_v02</t>
         </is>
       </c>
       <c r="E725" t="inlineStr">
@@ -35009,7 +35009,7 @@
       </c>
       <c r="G725" t="inlineStr">
         <is>
-          <t>02_Telegram/04_Эмодзи_Главная_группа/MOKO_18_эмодзи_группа_v01.zip</t>
+          <t>02_Telegram/04_Эмодзи_Главная_группа/MOKO_18_эмодзи_группа_v02.zip</t>
         </is>
       </c>
       <c r="H725" t="inlineStr">
@@ -35018,7 +35018,7 @@
         </is>
       </c>
       <c r="I725" t="n">
-        <v>573.5</v>
+        <v>489.6</v>
       </c>
     </row>
     <row r="726">
@@ -35034,7 +35034,7 @@
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
@@ -35058,7 +35058,7 @@
         </is>
       </c>
       <c r="I726" t="n">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="727">
@@ -35074,7 +35074,7 @@
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
@@ -35098,7 +35098,7 @@
         </is>
       </c>
       <c r="I727" t="n">
-        <v>182.1</v>
+        <v>169.4</v>
       </c>
     </row>
     <row r="728">
@@ -35114,7 +35114,7 @@
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
@@ -35154,7 +35154,7 @@
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>добавлено 18.09.2026 · не опубликовано</t>
+          <t>добавлено 18.09.2026 · v02 · не опубликовано</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
@@ -35178,7 +35178,7 @@
         </is>
       </c>
       <c r="I729" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>